<commit_message>
Replace survey-coding-sheet with updated version
</commit_message>
<xml_diff>
--- a/survey_coding_sheet_english.xlsx
+++ b/survey_coding_sheet_english.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Research_EC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0FDE206-17F0-4092-988E-B289B4A35EC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8940"/>
   </bookViews>
   <sheets>
     <sheet name="Variable_Mapping" sheetId="1" r:id="rId1"/>
@@ -1063,7 +1062,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1419,7 +1418,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1957,7 +1956,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2814,7 +2813,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2979,7 +2978,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>